<commit_message>
Updated Azure Deployment and Model
</commit_message>
<xml_diff>
--- a/outputs/coded_findings_verified.xlsx
+++ b/outputs/coded_findings_verified.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ecorys-my.sharepoint.com/personal/vincent_frippiat_ecorys_com/Documents/Documents/PnR/Sustainable Agriculture/PDF Processing Eleonora/lit_review/outputs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_0FE922F8EDC3C92CAD2C4C86F5EE235B78784956" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99960B13-0176-4150-A65A-61B93F84A14F}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="155">
   <si>
     <t>snippet_id</t>
   </si>
@@ -58,36 +64,6 @@
     <t>matched_text</t>
   </si>
   <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0001</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0002</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0003</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0004</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0005</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0006</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0007</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0008</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0009</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_EFFECTIVENESS__0010</t>
-  </si>
-  <si>
     <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_EFFECTIVENESS__0001</t>
   </si>
   <si>
@@ -136,31 +112,49 @@
     <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_EFFECTIVENESS__0016</t>
   </si>
   <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0001</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0002</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0003</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0004</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0005</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0006</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0007</t>
-  </si>
-  <si>
-    <t>AIPPI_position_paper_on_the_CPVO_CPVR_Ca__CPVR_LEGAL__0008</t>
-  </si>
-  <si>
-    <t>AIPPI position paper on the CPVO.CPVR Call for Evidence March 2025.pdf</t>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_EFFECTIVENESS__0017</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_EFFECTIVENESS__0018</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0001</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0002</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0003</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0004</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0005</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0006</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0007</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0008</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0009</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0010</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0011</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0012</t>
+  </si>
+  <si>
+    <t>Adelaiye__V_O___2024__Plant_Variety_Righ__CPVR_LEGAL__0013</t>
   </si>
   <si>
     <t>Adelaiye, V.O. (2024) Plant Variety Right and Intellectual Property Law in Nigeria A Review.pdf</t>
@@ -175,55 +169,43 @@
     <t>OBJECTIVES</t>
   </si>
   <si>
+    <t>INNOVATION_MARKET</t>
+  </si>
+  <si>
     <t>RIGHTS_BALANCE</t>
   </si>
   <si>
-    <t>INNOVATION_MARKET</t>
-  </si>
-  <si>
     <t>IP_FRAMEWORK</t>
   </si>
   <si>
     <t>IMPLEMENTATION_BARRIERS</t>
   </si>
   <si>
-    <t>Plant variety right protection is the most relevant form of intellectual property protection for plant varieties. To foster innovation in the field of plant breeding, the Basic Regulation should provide for strong and balanced IP protection for all stakeholders that invest in plant innovations, irrespective of how new plant varieties are developed, either by way of classic breeding and/or the use of new breeding technologies.</t>
-  </si>
-  <si>
-    <t>The interpretation given by the CJEU in its judgement of 19 December 2019 in the Nadorcott case (C-176 / 18) on unauthorized use of variety constituents in the context of provisional protection has a negative impact on the plant breeding industry in practice, especially in the field of ornamentals and fruit species.</t>
-  </si>
-  <si>
-    <t>The approach of the Court, that there is no unauthorized use of variety constituents if no authorization is required to propagate the material, limits the right to act against harvested material beyond the intentions of the UPOV legislator and has a chilling effect on the release of new plant varieties before the expiry of the provisional protection.</t>
-  </si>
-  <si>
-    <t>Holders of CPVR should have the same rights and remedies granted to other IP holders under the EU enforcement directive. To this end, the relation between the Basic Regulation and the EU enforcement directive should be clarified.</t>
-  </si>
-  <si>
-    <t>The definition of EDVs under Article 13(6), especially as regards the concepts of "predominantly derived" under Article 13(6)(a) and "conforms essentially to the initial variety in the expression of the characteristics …." under Article 13(6)(c), should be updated taking into account the guidance provided by the Explanatory Notes on Essentially Derived Varieties under the 1991 Act of the UPOV Convention, adopted by the Council at its fifty-seventh ordinary session on 27 October 2023 and further guidance should be provided on how to establish in practice if a variety is an EDV.</t>
-  </si>
-  <si>
-    <t>Article 95 provides that "Prior to the grant of Community plant variety rights, the holder may require reasonable compensation from any person who has, in the time between publication of the application for a Community plant variety right and grant thereof, effected an act that he would be prohibited from performing subsequent thereto". However, the concept of reasonable compensation is extremely vague and lends itself to different interpretations at the national level in the case of enforcement.</t>
-  </si>
-  <si>
-    <t>For provisional protection to be effective, it would be advisable to delineate the concept of "reasonable compensation" in its conceivable amount so as to provide reliable reference elements for (prospective) rights holders to prevent acts potentially adversely affecting their PVRs, where subsequently granted.</t>
-  </si>
-  <si>
-    <t>In Nigeria, the relationship between Plant Variety Protection (PVP) and traditional intellectual property rights (IPR) is evolving, especially with the recent enactment of the Plant Variety Protection Act in 2021 which aimed at: promoting increased staple crop productivity for smallholder farmers in Nigeria and encourage investment in plant breeding and crop variety development; promoting increased mutual accountability in the seed sector; and protecting new varieties of plants.</t>
+    <t>the recent enactment of the Plant Variety Protection Act in 2021 which aimed at: promoting increased staple crop productivity for smallholder farmers in Nigeria and encourage investment in plant breeding and crop variety development; promoting increased mutual accountability in the seed sector; and protecting new varieties of plants.</t>
   </si>
   <si>
     <t>Section 5 of the Plant Variety Protection Act 2021 established a Plant Variety Protection Office in Nigeria to grant breeders rights, facilitate transfer and licensing of plant breeder’s rights, collaborate with local and international bodies whose functions relate to plant breeding and perform other necessary functions.</t>
   </si>
   <si>
-    <t>PVR regimes, which are a part of larger IP regimes, seek to achieve a careful equilibrium between encouraging innovation and guaranteeing the preservation of genetic variation.</t>
-  </si>
-  <si>
-    <t>Fundamentally, PVR gives breeders an exclusive authority to commercially propagate, market, and distribute their registered plant varieties. PVR regimes encourage the generation of new varieties that are suited to address changing market needs and environmental issues by providing incentives for research and development.</t>
-  </si>
-  <si>
-    <t>However, the implementation of PVR regulations raises complex ethical, legal and socioeconomic considerations. Concerns about farmers' rights, benefit-sharing arrangements, and access to genetic resources are major problems that highlight the necessity of a comprehensive and inclusive approach to plant variety sustainability.</t>
-  </si>
-  <si>
-    <t>Nigeria was not a signatory to the International Union for the Protection of New Varieties of Plants (UPOV) Convention (Okonkwo, et al 2021) which to a large extent impeded the exploitation of such rights. It even deprived plant breeders in Nigeria access to high-quality new varieties of plant from foreign countries and also discourages foreign plant breeders since their new plant variety cannot be protected. These lacunae had surreptitiously deprived Nigeria of innovative opportunities in this sector unlike her counterparts – Uganda (Uganda Plant Variety Act2014), Kenya (Seed and Plant Varieties Act 2012) and South Africa (Plant Breeder’s Rights Act 1976).</t>
+    <t>This includes monitoring the market for potential infringements and taking legal action against unauthorized use of protected varieties. Breeders can also seek legal remedies through the courts if their rights are violated</t>
+  </si>
+  <si>
+    <t>The PVP Act grants registered plant breeders Intellectual Property rights, thereby providing incentives for the development of new crop varieties and encouraging more farmers to engage in plant breeding.</t>
+  </si>
+  <si>
+    <t>It is expected that the proper implementation of the provisions of the PVP will encourage research and development by breeders, thereby leading to higher agricultural productivity, and a boost in the agricultural sector would have a reverberating effect on Nigeria’s economy.</t>
+  </si>
+  <si>
+    <t>The Registrar should make effective guidelines for the effective implementation of the Act.</t>
+  </si>
+  <si>
+    <t>This will endeavour that NASC can handle applications, conduct examinations and enforce rights where necessary.</t>
+  </si>
+  <si>
+    <t>PVR regimes encourage the generation of new varieties that are suited to address changing market needs and environmental issues by providing incentives for research and development.</t>
+  </si>
+  <si>
+    <t>Nigeria was not a signatory to the International Union for the Protection of New Varieties of Plants (UPOV) Convention (Okonkwo, et al 2021) which to a large extent impeded the exploitation of such rights. It even deprived plant breeders in Nigeria access to high-quality new varieties of plant from foreign countries and also discourages foreign plant breeders since their new plant variety cannot be protected.</t>
   </si>
   <si>
     <t>Comparing plant variety systems in other countries, it's evident that regulatory frameworks and breeder rights are crucial for fully exploiting breeding activities, as new plant varieties require significant investment in skills, labor, resources, and time. Intellectual property (IP) protection is, therefore, necessary to serve as an incentive to plant breeders, for the development of new varieties to contribute to sustainable progress in agriculture.</t>
@@ -232,151 +214,154 @@
     <t>This system encourages investment in plant breeding and crop variety development, aiming to boost agricultural productivity and innovation.</t>
   </si>
   <si>
+    <t>Intellectual Property protection for plant breeders boosts investment in breeding and developing new plant varieties, as investors can now rely on a structured protection system.</t>
+  </si>
+  <si>
+    <t>The PVP Act will encourage non-resident or foreign plant breeder applications, enhancing access to foreign plant varieties by ensuring adequate protection of their varieties.</t>
+  </si>
+  <si>
+    <t>Concerns about farmers' rights, benefit-sharing arrangements, and access to genetic resources are major problems that highlight the necessity of a comprehensive and inclusive approach to plant variety sustainability.</t>
+  </si>
+  <si>
     <t>Breeders have the right to save seeds for the future use to the exclusion of other farmers within a reasonable limit and subject to the safeguarding of the interest of the breeders(Article 15(2) of UPOV).</t>
   </si>
   <si>
-    <t>A plant breeder has exclusive rights to propagate materials of a protected variety. Authorization must be obtained from such a breeder for the production and reproduction, conditioning for propagation; offering for sale; selling or marketing; exporting; importing and stocking in relation to any of the mentioned purposes. Any authorization given by the plant breeder may be subject to conditions and limitations. However, such exclusive rights of a plant breeder cannot impede the doing of the following acts by a third party without authorization: Private and non-commercial purposes; Experimental purposes; and for the purpose of breeding any other variety, except it is essentially derived from an initially protected variety.</t>
-  </si>
-  <si>
-    <t>1. The PVP Act grants registered plant breeders Intellectual Property rights, thereby providing incentives for the development of new crop varieties and encouraging more farmers to engage in plant breeding.</t>
-  </si>
-  <si>
-    <t>3. Intellectual Property protection for plant breeders boosts investment in breeding and developing new plant varieties, as investors can now rely on a structured protection system.</t>
-  </si>
-  <si>
-    <t>4. The PVP Act will encourage non-resident or foreign plant breeder applications, enhancing access to foreign plant varieties by ensuring adequate protection of their varieties.</t>
-  </si>
-  <si>
-    <t>5. It is expected that the proper implementation of the provisions of the PVP will encourage research and development by breeders, thereby leading to higher agricultural productivity, and a boost in the agricultural sector would have a reverberating effect on Nigeria’s economy.</t>
-  </si>
-  <si>
-    <t>The passing of the Plant Protection Variety Act heralded numerous opportunities in the agricultural sector as plant breeders can commercialize their intellectual property by assigning or authorizing any activity in relation to any registered plant variety. This also opens investment opportunities for investors seeking to explore this aspect of agriculture and further creates job opportunities for people skilled in agriculture.</t>
-  </si>
-  <si>
-    <t>To ensure breeders can benefit from the full scope of protection provided for under UPOV 1991 and to make the system future-proof in view of technical progress in plant breeding, the Basic Regulation and related regulations should be improved and clarified</t>
-  </si>
-  <si>
-    <t>Trigger exhaustion (Article 16 Basic Regulation). The wording of the trigger for exhaustion in Article 16 Basic Regulation (disposed of to others) deviates from the wording used in Article 16 UPOV 1991 (sold or otherwise marketed). The trigger for exhaustion should be clarified.</t>
-  </si>
-  <si>
-    <t>Enforcement. Holders of CPVR should have the same rights and remedies granted to other IP holders under the EU enforcement directive. To this end, the relation between the Basic Regulation and the EU enforcement directive should be clarified.</t>
-  </si>
-  <si>
-    <t>Furthermore, cost-efficient enforcement measures should be available for breeders to act against unauthorized use of protected plant material and harvested material.</t>
-  </si>
-  <si>
-    <t>Essentially Derived Varieties - EDVs (Article 13(6), Basic Regulation). The definition of EDVs under Article 13(6), especially as regards the concepts of "predominantly derived" under Article 13(6)(a) and "conforms essentially to the initial variety in the expression of the characteristics …." under Article 13(6)(c), should be updated taking into account the guidance provided by the Explanatory Notes on Essentially Derived Varieties under the 1991 Act of the UPOV Convention, adopted by the Council at its fifty-seventh ordinary session on 27 October 2023</t>
-  </si>
-  <si>
-    <t>Variety Denominations (Article 17, Basic Regulation). Under the terms of Article 17, the obligations relating to the use of the variety denominations contained in paragraphs 1 and 2 "shall apply even after the termination of the Community plant variety right". However, it is unclear who is entitled to enforce the related rights after the PVR expiry, and by which means.</t>
-  </si>
-  <si>
-    <t>Provisional protection (Article 95, Basic Regulation). Article 95 provides that "Prior to the grant of Community plant variety rights, the holder may require reasonable compensation from any person who has, in the time between publication of the application for a Community plant variety right and grant thereof, effected an act that he would be prohibited from performing subsequent thereto". However, the concept of reasonable compensation is extremely vague and lends itself to different interpretations at the national level in the case of enforcement.</t>
-  </si>
-  <si>
-    <t>A harmonization of terminology with the UPOV Convention might be advisable as well as the inclusion of a specific article providing for basic definitions.</t>
-  </si>
-  <si>
-    <t>This passage explicitly states policy goals for the Basic Regulation, including fostering innovation and providing balanced protection.</t>
-  </si>
-  <si>
-    <t>The phrase "strong and balanced IP protection for all stakeholders" directly concerns balancing rights within the CPVR framework.</t>
-  </si>
-  <si>
-    <t>This passage directly links CPVR to innovation in plant breeding and investment in plant innovations.</t>
-  </si>
-  <si>
-    <t>This passage discusses a concrete impact of CPVR interpretation on the plant breeding industry, relevant to innovation and competitiveness.</t>
-  </si>
-  <si>
-    <t>This passage concerns the scope of breeders' rights and limitations on enforcing those rights under CPVR.</t>
-  </si>
-  <si>
-    <t>The reference to a "chilling effect on the release of new plant varieties" directly concerns innovation outcomes and market introduction.</t>
-  </si>
-  <si>
-    <t>This passage directly addresses the rights and remedies available to CPVR holders within the legal regime.</t>
-  </si>
-  <si>
-    <t>This concerns the EDV framework, which is closely tied to breeding activity, varietal development, and competitive innovation conditions.</t>
-  </si>
-  <si>
-    <t>This passage addresses provisional protection and compensation, which are core elements of the balance and enforceability of breeders' rights.</t>
-  </si>
-  <si>
-    <t>This directly concerns strengthening and clarifying legal protections for rights holders under CPVR.</t>
-  </si>
-  <si>
-    <t>This passage explicitly states the aims of the 2021 Act, directly matching legislative and policy objectives.</t>
-  </si>
-  <si>
-    <t>This describes institutional functions under the Act, including oversight and administration relevant to CPVR-type objectives and implementation.</t>
-  </si>
-  <si>
-    <t>This directly links plant variety rights to encouraging innovation.</t>
-  </si>
-  <si>
-    <t>This passage addresses both innovation outcomes and market aspects, including commercialization and incentives for developing new varieties.</t>
-  </si>
-  <si>
-    <t>This explicitly discusses farmers' rights and related balancing considerations within the PVR framework.</t>
-  </si>
-  <si>
-    <t>This passage links plant variety protection to innovation opportunities, access to foreign varieties, and breeder participation in the market.</t>
-  </si>
-  <si>
-    <t>This directly discusses breeding activity, incentives, and development of new varieties as innovation outcomes.</t>
-  </si>
-  <si>
-    <t>This states intended outcomes of the protection system, aligning with legislative and policy objectives.</t>
-  </si>
-  <si>
-    <t>This passage clearly addresses innovation and breeding investment impacts.</t>
-  </si>
-  <si>
-    <t>This passage directly concerns the balance between breeders' interests and seed-saving/farmer-related exceptions under the legal framework.</t>
-  </si>
-  <si>
-    <t>This passage clearly sets out breeders' exclusive rights alongside exceptions, showing the legal balance of rights and limitations.</t>
-  </si>
-  <si>
-    <t>This directly links the Act to incentives for developing new varieties and increasing breeding activity.</t>
-  </si>
-  <si>
-    <t>This explicitly addresses investment and development of new varieties, central to innovation and market effects.</t>
-  </si>
-  <si>
-    <t>This passage is about market access and cross-border breeder participation resulting from protection.</t>
-  </si>
-  <si>
-    <t>This directly concerns R&amp;D by breeders and broader economic and innovation-related effects.</t>
-  </si>
-  <si>
-    <t>This passage discusses commercialization, investment opportunities, and sectoral economic effects, all relevant to innovation and market impact.</t>
-  </si>
-  <si>
-    <t>Directly references alignment of the Basic Regulation with UPOV 1991, which fits the international IP framework label.</t>
-  </si>
-  <si>
-    <t>Explicit comparison between the CPVR Basic Regulation and UPOV 1991 shows interaction with an international IP standard.</t>
-  </si>
-  <si>
-    <t>Directly addresses how CPVR interacts with the EU IP enforcement framework.</t>
-  </si>
-  <si>
-    <t>This points to enforcement availability as an implementation issue affecting operational effectiveness of CPVR.</t>
-  </si>
-  <si>
-    <t>References the UPOV Convention as guidance for updating CPVR rules, fitting international IP alignment.</t>
-  </si>
-  <si>
-    <t>Highlights ambiguity in enforcement responsibility and means, which is a barrier to implementation.</t>
-  </si>
-  <si>
-    <t>Describes vagueness and divergent national interpretations in enforcement, a clear implementation barrier.</t>
-  </si>
-  <si>
-    <t>Explicitly calls for harmonization with the UPOV Convention, directly matching the international IP framework label.</t>
+    <t>Any authorization given by the plant breeder may be subject to conditions and limitations. However, such exclusive rights of a plant breeder cannot impede the doing of the following acts by a third party without authorization: Private and non-commercial purposes; Experimental purposes; and for the purpose of breeding any other variety, except it is essentially derived from an initially protected variety.</t>
+  </si>
+  <si>
+    <t>The Plant Variety Protection Act 2021 established a Plant Variety Protection Office in Nigeria to grant breeders rights, facilitate transfer and licensing of plant breeder’s rights</t>
+  </si>
+  <si>
+    <t>The Plant Variety Protection Act 2021 makes provision for the holder of a plant breeder’s right to assign or authorize any activity in relation to a registered plant variety.</t>
+  </si>
+  <si>
+    <t>Recognizing the importance of Plant Variety Right and Intellectual Property Law in Nigeria: A Review harmonizing plant variety protection laws to facilitate international trade in plant germplasm and promote agricultural innovation, efforts were made to establish international agreements in this area. One of the most significant developments was the adoption of the International Union for the Protection of New Plant Varieties Convention (UPOV Convention) in 1961.</t>
+  </si>
+  <si>
+    <t>Nigeria was not a signatory to the International Union for the Protection of New Varieties of Plants (UPOV) Convention (Okonkwo, et al 2021) which to a large extent impeded the exploitation of such rights.</t>
+  </si>
+  <si>
+    <t>Meanwhile, the Trade-Related Aspects of Intellectual Property Rights Agreement (TRIPS), which Nigeria is a signatory to, recognizes and provides for the patentability of inventions in all fields of technology and specifically calls for the protection of plant varieties either by patent or by an effective sui generis system or by any combination thereof in line with the provisions of Article 27 of the TRIPS Agreement.</t>
+  </si>
+  <si>
+    <t>Some African countries have opted for the adoption of the International Convention for the Protection of New Varieties of Plants (UPOV Convention) while others have enacted a sui generis plant variety protection law.</t>
+  </si>
+  <si>
+    <t>The Act aligns with international standards, such as those set by the International Union for the Protection of New Varieties of Plants (UPOV).</t>
+  </si>
+  <si>
+    <t>In some jurisdictions like the United State and Australia, the subject matter of protection covered by a Traditional IP and by a plant breeder’s right might be the same, namely a plant variety while in several other jurisdictions like European Union and India, the subject matter of protection is different, and, in general, plant varieties are excluded from patentability.</t>
+  </si>
+  <si>
+    <t>As far as the International Union for the Protection of New Plant Varieties Convention (UPOV) is concerned, a member is free to protect plant varieties, in addition to the grant of a breeder’s right, by the grant of other titles, particularly patents.</t>
+  </si>
+  <si>
+    <t>TRIPS do not specify detailed criteria for plant variety protection but requires member countries to establish effective systems for the protection of plant varieties.</t>
+  </si>
+  <si>
+    <t>It allows flexibility for countries to determine their own criteria, which may include patent, or by an effective sui generis system (which could be UPOV standards) or by combination of both systems.</t>
+  </si>
+  <si>
+    <t>The National Agricultural Seeds Council (NASC) should be given adequate resources and trained personnel to effectively manage the PVP system. This will endeavour that NASC can handle applications, conduct examinations and enforce rights where necessary.</t>
+  </si>
+  <si>
+    <t>A well structured awareness program could be implemented at all level of the society to sensitize farmers, breeders, legislators and the general public on the intellectual property rights and plant variety rights and how they support innovation and food security.</t>
+  </si>
+  <si>
+    <t>Regular monitoring of the market for unauthorized use or infringement on plant varieties. Prompt action should be taken to enforce intellectual property rights through legal means such as sending cease-and-desist letters or pursuing litigation.</t>
+  </si>
+  <si>
+    <t>This passage explicitly states the legislative and policy objectives of Nigeria’s Plant Variety Protection Act.</t>
+  </si>
+  <si>
+    <t>This directly addresses the institutional framework and oversight functions established to implement the plant variety protection system.</t>
+  </si>
+  <si>
+    <t>The passage describes enforcement and monitoring activities supporting the legislative objective of protecting plant breeders’ rights.</t>
+  </si>
+  <si>
+    <t>This identifies an intended performance outcome of the Act: incentivising new variety development and broader breeding activity.</t>
+  </si>
+  <si>
+    <t>This links implementation of the plant variety protection framework to its intended objectives of research, productivity, and economic development.</t>
+  </si>
+  <si>
+    <t>This recommendation concerns effective implementation of the core plant variety protection legislation.</t>
+  </si>
+  <si>
+    <t>The passage directly addresses administrative oversight of applications, examination, and enforcement within the plant variety protection system.</t>
+  </si>
+  <si>
+    <t>This explicitly connects plant variety rights with breeding innovation and responsiveness to market needs.</t>
+  </si>
+  <si>
+    <t>This passage addresses the effects of the protection regime on access to varieties, foreign breeding activity, and exploitation of plant breeding rights.</t>
+  </si>
+  <si>
+    <t>The passage directly links plant variety protection to breeding investment, exploitation of breeding activities, and development of new varieties.</t>
+  </si>
+  <si>
+    <t>This explicitly describes the expected innovation and productivity effects of the plant variety protection system.</t>
+  </si>
+  <si>
+    <t>This passage addresses the relationship between plant variety protection, investment, and varietal innovation.</t>
+  </si>
+  <si>
+    <t>This directly concerns market access to foreign varieties and the effect of protection on international breeding activity.</t>
+  </si>
+  <si>
+    <t>This explicitly identifies farmers’ rights and benefit sharing as considerations that must be balanced within the plant variety protection system.</t>
+  </si>
+  <si>
+    <t>This directly addresses the relationship between breeders’ seed-saving rights and the interests of farmers.</t>
+  </si>
+  <si>
+    <t>This passage defines limitations and exceptions to breeders’ exclusive rights, including private, experimental, and further-breeding uses.</t>
+  </si>
+  <si>
+    <t>This directly addresses the licensing regime and administration of breeders’ rights under the plant variety protection framework.</t>
+  </si>
+  <si>
+    <t>This passage concerns the legal mechanisms for assignment and authorization of activities involving protected varieties.</t>
+  </si>
+  <si>
+    <t>This passage directly discusses the international harmonization of plant variety protection through the UPOV Convention.</t>
+  </si>
+  <si>
+    <t>The passage explicitly addresses Nigeria’s relationship with UPOV and the consequences of non-alignment with that international IP system.</t>
+  </si>
+  <si>
+    <t>This passage directly explains Nigeria’s obligations under TRIPS concerning plant variety protection.</t>
+  </si>
+  <si>
+    <t>The passage compares UPOV-based protection with national sui generis systems, directly addressing interaction between international and domestic IP frameworks.</t>
+  </si>
+  <si>
+    <t>This is a direct statement about alignment between Nigeria’s Plant Variety Protection Act and UPOV standards.</t>
+  </si>
+  <si>
+    <t>This passage explicitly references the European Union framework and compares plant variety rights with traditional IP protection.</t>
+  </si>
+  <si>
+    <t>The passage directly explains how UPOV interacts with other IP titles, particularly patents.</t>
+  </si>
+  <si>
+    <t>This passage describes the relationship between TRIPS obligations and national plant variety protection systems.</t>
+  </si>
+  <si>
+    <t>This directly addresses how TRIPS permits countries to implement plant variety protection through patents, sui generis systems, UPOV standards, or combinations thereof.</t>
+  </si>
+  <si>
+    <t>The passage identifies non-participation in UPOV and the resulting lack of protection and access as barriers to effective implementation and exploitation of plant variety rights.</t>
+  </si>
+  <si>
+    <t>This explicitly identifies inadequate resources and trained personnel as capacity barriers affecting administration, examination, and enforcement of the PVP system.</t>
+  </si>
+  <si>
+    <t>The recommendation indicates a knowledge and awareness gap among key stakeholders that may hinder compliance with and implementation of plant variety rights.</t>
+  </si>
+  <si>
+    <t>This passage addresses enforcement needs, including market monitoring and prompt action against unauthorized use or infringement.</t>
   </si>
   <si>
     <t>high</t>
@@ -385,125 +370,128 @@
     <t>medium</t>
   </si>
   <si>
-    <t>2026-07-09T13:57:31</t>
-  </si>
-  <si>
-    <t>2026-07-09T13:57:52</t>
-  </si>
-  <si>
-    <t>4885febfda356ba8</t>
-  </si>
-  <si>
-    <t>db560946c5a52cd1</t>
-  </si>
-  <si>
-    <t>0b0cda6ea456ae18</t>
-  </si>
-  <si>
-    <t>98bededa55afd02f</t>
-  </si>
-  <si>
-    <t>f0dd8fa3e5752042</t>
-  </si>
-  <si>
-    <t>72026d02c929d901</t>
-  </si>
-  <si>
-    <t>e1e2caa33ec59a34</t>
-  </si>
-  <si>
-    <t>b8687c2ff2bbad02</t>
-  </si>
-  <si>
-    <t>d975bc2534fd8579</t>
-  </si>
-  <si>
-    <t>1f3cc95cab3d84c6</t>
-  </si>
-  <si>
-    <t>a15be750d6e0dcbd</t>
+    <t>2026-07-13T10:46:49</t>
+  </si>
+  <si>
+    <t>2026-07-13T10:46:59</t>
+  </si>
+  <si>
+    <t>921c44f647cb8414</t>
   </si>
   <si>
     <t>0a0c5adc352ca23e</t>
   </si>
   <si>
-    <t>bdc4a4c520252ed4</t>
-  </si>
-  <si>
-    <t>27957cdc75878627</t>
-  </si>
-  <si>
-    <t>aa25b5fbb0c63bc9</t>
-  </si>
-  <si>
-    <t>62cf06fc8b087b12</t>
+    <t>15d08dae243bf0dd</t>
+  </si>
+  <si>
+    <t>e62fa8101dcbf495</t>
+  </si>
+  <si>
+    <t>8ab423e4f332419c</t>
+  </si>
+  <si>
+    <t>336157c31767af2e</t>
+  </si>
+  <si>
+    <t>c64f3b49bdbdbda6</t>
+  </si>
+  <si>
+    <t>60d3fa74711ddeff</t>
+  </si>
+  <si>
+    <t>0399a0f00984de28</t>
   </si>
   <si>
     <t>6d1276c2c269771d</t>
   </si>
   <si>
-    <t>a17bedcc73b313ea</t>
-  </si>
-  <si>
     <t>e25cc72fd7fe642d</t>
   </si>
   <si>
+    <t>0006dfdbe2556ca6</t>
+  </si>
+  <si>
+    <t>e26a5410d9566630</t>
+  </si>
+  <si>
+    <t>ea8f818b2d551ebe</t>
+  </si>
+  <si>
     <t>304d5e591be7ff7c</t>
   </si>
   <si>
-    <t>93ef8e4a617899b8</t>
-  </si>
-  <si>
-    <t>c385ada89e152b2a</t>
-  </si>
-  <si>
-    <t>3bdd9b777dc8ddd5</t>
-  </si>
-  <si>
-    <t>b49ca5012f68706e</t>
-  </si>
-  <si>
-    <t>388aa1a7a82d4eb6</t>
-  </si>
-  <si>
-    <t>12ce00b83501e378</t>
-  </si>
-  <si>
-    <t>78ca97f356748bd0</t>
-  </si>
-  <si>
-    <t>60826a686b8efa72</t>
-  </si>
-  <si>
-    <t>e5907597a32b23e5</t>
-  </si>
-  <si>
-    <t>4aeae4ca4140550c</t>
-  </si>
-  <si>
-    <t>3992db46e85ec29d</t>
-  </si>
-  <si>
-    <t>fb665a95cd9a7236</t>
-  </si>
-  <si>
-    <t>6216360d628f61d6</t>
-  </si>
-  <si>
-    <t>26bd3ff19bf9afcd</t>
+    <t>bed60198aa7d98d7</t>
+  </si>
+  <si>
+    <t>293bedc63ccac696</t>
+  </si>
+  <si>
+    <t>b8b95517fe0ec991</t>
+  </si>
+  <si>
+    <t>6e75c954be94e497</t>
+  </si>
+  <si>
+    <t>981ccf352303e94c</t>
+  </si>
+  <si>
+    <t>c610e80e31bf16e2</t>
+  </si>
+  <si>
+    <t>1241964aeb0d668a</t>
+  </si>
+  <si>
+    <t>f2a89608af05241d</t>
+  </si>
+  <si>
+    <t>b498bb48c3975e6e</t>
+  </si>
+  <si>
+    <t>d45207dcc9ebd233</t>
+  </si>
+  <si>
+    <t>81970ea37993455b</t>
+  </si>
+  <si>
+    <t>78836028559f5700</t>
+  </si>
+  <si>
+    <t>7dda530f2181d6e8</t>
+  </si>
+  <si>
+    <t>952879e5e9fdd222</t>
+  </si>
+  <si>
+    <t>7d12f70da1199b71</t>
+  </si>
+  <si>
+    <t>08fe648d8f55b74f</t>
   </si>
   <si>
     <t>verified</t>
   </si>
   <si>
+    <t>near_match</t>
+  </si>
+  <si>
+    <t>verified_fuzzy</t>
+  </si>
+  <si>
     <t>exact</t>
+  </si>
+  <si>
+    <t>fuzzy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regular monitoring of the market for unauthorized use or infringement on plant varieties. Prompt action should be taken to enforce intellectual property rights through legal means such as sending cease-anddesist letters or pursuing litigation. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -566,13 +554,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -610,7 +606,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -644,6 +640,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -678,9 +675,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -853,11 +851,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N35"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N32"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -901,1398 +899,1278 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
         <v>48</v>
       </c>
-      <c r="C2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" t="s">
-        <v>52</v>
-      </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="H2" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="K2" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L2">
         <v>100</v>
       </c>
       <c r="M2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
         <v>48</v>
       </c>
-      <c r="C3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" t="s">
-        <v>53</v>
-      </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="H3" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I3" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J3" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="K3" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L3">
         <v>100</v>
       </c>
       <c r="M3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
         <v>48</v>
       </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" t="s">
-        <v>54</v>
-      </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H4" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I4" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J4" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="K4" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L4">
         <v>100</v>
       </c>
       <c r="M4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
       <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
         <v>48</v>
       </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" t="s">
-        <v>54</v>
-      </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I5" t="s">
+        <v>116</v>
+      </c>
+      <c r="J5" t="s">
         <v>121</v>
       </c>
-      <c r="I5" t="s">
-        <v>123</v>
-      </c>
-      <c r="J5" t="s">
-        <v>128</v>
-      </c>
       <c r="K5" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L5">
         <v>100</v>
       </c>
       <c r="M5" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
       <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
         <v>48</v>
       </c>
-      <c r="C6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" t="s">
-        <v>53</v>
-      </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H6" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I6" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J6" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="K6" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L6">
         <v>100</v>
       </c>
       <c r="M6" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" t="s">
-        <v>54</v>
-      </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H7" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I7" t="s">
+        <v>116</v>
+      </c>
+      <c r="J7" t="s">
         <v>123</v>
       </c>
-      <c r="J7" t="s">
-        <v>130</v>
-      </c>
       <c r="K7" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L7">
         <v>100</v>
       </c>
       <c r="M7" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>20</v>
       </c>
       <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" t="s">
-        <v>53</v>
-      </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H8" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I8" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J8" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="K8" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L8">
         <v>100</v>
       </c>
       <c r="M8" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="H9" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="I9" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J9" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="K9" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L9">
         <v>100</v>
       </c>
       <c r="M9" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="H10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I10" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J10" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="K10" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L10">
         <v>100</v>
       </c>
       <c r="M10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G11" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="H11" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I11" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J11" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="K11" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L11">
         <v>100</v>
       </c>
       <c r="M11" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>24</v>
       </c>
       <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
         <v>49</v>
       </c>
-      <c r="C12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
-      </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F12">
         <v>4</v>
       </c>
       <c r="G12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H12" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I12" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J12" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="K12" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L12">
         <v>100</v>
       </c>
       <c r="M12" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
       <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
         <v>49</v>
       </c>
-      <c r="C13" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" t="s">
-        <v>52</v>
-      </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F13">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="H13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I13" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J13" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="K13" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L13">
         <v>100</v>
       </c>
       <c r="M13" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
       <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
         <v>49</v>
       </c>
-      <c r="C14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" t="s">
-        <v>54</v>
-      </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H14" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I14" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J14" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K14" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L14">
         <v>100</v>
       </c>
       <c r="M14" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
         <v>50</v>
       </c>
-      <c r="D15" t="s">
-        <v>54</v>
-      </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H15" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I15" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J15" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="K15" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L15">
         <v>100</v>
       </c>
       <c r="M15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
         <v>50</v>
       </c>
-      <c r="D16" t="s">
-        <v>53</v>
-      </c>
       <c r="E16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G16" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H16" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I16" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J16" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="K16" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L16">
         <v>100</v>
       </c>
       <c r="M16" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
         <v>50</v>
       </c>
-      <c r="D17" t="s">
-        <v>54</v>
-      </c>
       <c r="E17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F17">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G17" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H17" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I17" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J17" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="K17" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L17">
         <v>100</v>
       </c>
       <c r="M17" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" t="s">
         <v>50</v>
       </c>
-      <c r="D18" t="s">
-        <v>54</v>
-      </c>
       <c r="E18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F18">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H18" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I18" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J18" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="K18" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L18">
         <v>100</v>
       </c>
       <c r="M18" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
         <v>50</v>
       </c>
-      <c r="D19" t="s">
-        <v>52</v>
-      </c>
       <c r="E19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G19" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="H19" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I19" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J19" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="K19" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L19">
         <v>100</v>
       </c>
       <c r="M19" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>32</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D20" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E20" t="s">
         <v>71</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H20" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I20" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J20" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="K20" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="L20">
-        <v>100</v>
+        <v>88.4</v>
       </c>
       <c r="M20" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E21" t="s">
         <v>72</v>
       </c>
       <c r="F21">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G21" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H21" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="I21" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J21" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="K21" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L21">
         <v>100</v>
       </c>
       <c r="M21" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E22" t="s">
         <v>73</v>
       </c>
       <c r="F22">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G22" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H22" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I22" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J22" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="K22" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L22">
         <v>100</v>
       </c>
       <c r="M22" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E23" t="s">
         <v>74</v>
       </c>
       <c r="F23">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G23" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I23" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J23" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="K23" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L23">
         <v>100</v>
       </c>
       <c r="M23" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E24" t="s">
         <v>75</v>
       </c>
       <c r="F24">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H24" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I24" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J24" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="K24" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L24">
         <v>100</v>
       </c>
       <c r="M24" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>37</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E25" t="s">
         <v>76</v>
       </c>
       <c r="F25">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G25" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="H25" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I25" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J25" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="K25" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L25">
         <v>100</v>
       </c>
       <c r="M25" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>38</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E26" t="s">
         <v>77</v>
       </c>
       <c r="F26">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G26" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H26" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I26" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J26" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="K26" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L26">
         <v>100</v>
       </c>
       <c r="M26" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E27" t="s">
         <v>78</v>
       </c>
       <c r="F27">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G27" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H27" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I27" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="J27" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="K27" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L27">
         <v>100</v>
       </c>
       <c r="M27" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" t="s">
         <v>51</v>
-      </c>
-      <c r="D28" t="s">
-        <v>55</v>
       </c>
       <c r="E28" t="s">
         <v>79</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G28" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H28" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I28" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J28" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="K28" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L28">
         <v>100</v>
       </c>
       <c r="M28" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>41</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D29" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E29" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G29" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H29" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I29" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J29" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="K29" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L29">
         <v>100</v>
       </c>
       <c r="M29" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>42</v>
       </c>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D30" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F30">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G30" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H30" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="I30" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J30" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="K30" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L30">
         <v>100</v>
       </c>
       <c r="M30" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>43</v>
       </c>
       <c r="B31" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C31" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D31" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="G31" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H31" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="I31" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J31" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="K31" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L31">
         <v>100</v>
       </c>
       <c r="M31" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>44</v>
       </c>
       <c r="B32" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C32" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D32" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G32" t="s">
+        <v>113</v>
+      </c>
+      <c r="H32" t="s">
+        <v>114</v>
+      </c>
+      <c r="I32" t="s">
         <v>117</v>
       </c>
-      <c r="H32" t="s">
-        <v>121</v>
-      </c>
-      <c r="I32" t="s">
-        <v>124</v>
-      </c>
       <c r="J32" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="K32" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="L32">
-        <v>100</v>
+        <v>99.6</v>
       </c>
       <c r="M32" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13">
-      <c r="A33" t="s">
-        <v>45</v>
-      </c>
-      <c r="B33" t="s">
-        <v>48</v>
-      </c>
-      <c r="C33" t="s">
-        <v>51</v>
-      </c>
-      <c r="D33" t="s">
-        <v>56</v>
-      </c>
-      <c r="E33" t="s">
-        <v>84</v>
-      </c>
-      <c r="F33">
-        <v>2</v>
-      </c>
-      <c r="G33" t="s">
-        <v>118</v>
-      </c>
-      <c r="H33" t="s">
-        <v>121</v>
-      </c>
-      <c r="I33" t="s">
-        <v>124</v>
-      </c>
-      <c r="J33" t="s">
-        <v>156</v>
-      </c>
-      <c r="K33" t="s">
-        <v>159</v>
-      </c>
-      <c r="L33">
-        <v>100</v>
-      </c>
-      <c r="M33" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13">
-      <c r="A34" t="s">
-        <v>46</v>
-      </c>
-      <c r="B34" t="s">
-        <v>48</v>
-      </c>
-      <c r="C34" t="s">
-        <v>51</v>
-      </c>
-      <c r="D34" t="s">
-        <v>56</v>
-      </c>
-      <c r="E34" t="s">
-        <v>85</v>
-      </c>
-      <c r="F34">
-        <v>2</v>
-      </c>
-      <c r="G34" t="s">
-        <v>119</v>
-      </c>
-      <c r="H34" t="s">
-        <v>121</v>
-      </c>
-      <c r="I34" t="s">
-        <v>124</v>
-      </c>
-      <c r="J34" t="s">
-        <v>157</v>
-      </c>
-      <c r="K34" t="s">
-        <v>159</v>
-      </c>
-      <c r="L34">
-        <v>100</v>
-      </c>
-      <c r="M34" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13">
-      <c r="A35" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" t="s">
-        <v>48</v>
-      </c>
-      <c r="C35" t="s">
-        <v>51</v>
-      </c>
-      <c r="D35" t="s">
-        <v>55</v>
-      </c>
-      <c r="E35" t="s">
-        <v>86</v>
-      </c>
-      <c r="F35">
-        <v>2</v>
-      </c>
-      <c r="G35" t="s">
-        <v>120</v>
-      </c>
-      <c r="H35" t="s">
-        <v>121</v>
-      </c>
-      <c r="I35" t="s">
-        <v>124</v>
-      </c>
-      <c r="J35" t="s">
-        <v>158</v>
-      </c>
-      <c r="K35" t="s">
-        <v>159</v>
-      </c>
-      <c r="L35">
-        <v>100</v>
-      </c>
-      <c r="M35" t="s">
-        <v>160</v>
+        <v>153</v>
+      </c>
+      <c r="N32" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>